<commit_message>
Implemented methods for calculating cover crop area and residues
</commit_message>
<xml_diff>
--- a/data/default/CoverCropsMgmt.xlsx
+++ b/data/default/CoverCropsMgmt.xlsx
@@ -153,6 +153,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -211,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -221,6 +224,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -858,7 +862,7 @@
       <c r="D25" t="s">
         <v>22</v>
       </c>
-      <c r="E25">
+      <c r="E25" s="9">
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="F25" t="s">
@@ -913,7 +917,7 @@
       <c r="D30" t="s">
         <v>22</v>
       </c>
-      <c r="E30">
+      <c r="E30" s="9">
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="F30" t="s">

</xml_diff>

<commit_message>
Pars. for rhizodeposited C and Jcobs bg_resid not to include rhizodep.
</commit_message>
<xml_diff>
--- a/data/default/CoverCropsMgmt.xlsx
+++ b/data/default/CoverCropsMgmt.xlsx
@@ -1,30 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E80A0529-2F6E-483A-9BEB-62AFB360DAE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6900"/>
+    <workbookView xWindow="-25080" yWindow="4380" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="60">
   <si>
     <t>parameter</t>
   </si>
@@ -146,9 +158,6 @@
     <t>Carbon in cover crop biomass</t>
   </si>
   <si>
-    <t>These parameters are not used at the moment…</t>
-  </si>
-  <si>
     <t>8 Övre Norrland</t>
   </si>
   <si>
@@ -188,24 +197,36 @@
     <t>soil_loss_adjust</t>
   </si>
   <si>
-    <t>The leaching/soil losses of the crop succeeding the cover crop is multiplied by the corresponding factor factor. A factor of 1 means no effect of cover crop</t>
-  </si>
-  <si>
     <t>and a factor lower than 1 means that leaching/soil losses are reduced.</t>
   </si>
   <si>
     <t>Note: This is not ideal as it is rather leaching/soil losses from the preceding crop that are reduced</t>
+  </si>
+  <si>
+    <t>rhizodep_C</t>
+  </si>
+  <si>
+    <t>kg C/kg C</t>
+  </si>
+  <si>
+    <t>Rhizodeposited C in relation to below ground biomass C</t>
+  </si>
+  <si>
+    <t>Bolinder et al. 2007</t>
+  </si>
+  <si>
+    <t>The leaching/soil losses of the crop succeeding the cover crop is multiplied by the corresponding factor. A factor of 1 means no effect of cover crop</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -249,14 +270,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -284,7 +297,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -296,14 +309,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -583,8 +594,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I116"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I117"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -628,7 +639,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="6"/>
@@ -675,7 +686,7 @@
       <c r="C6" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" t="s">
         <v>28</v>
       </c>
       <c r="E6" t="s">
@@ -689,10 +700,10 @@
         <v>5</v>
       </c>
       <c r="H6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I6" t="s">
         <v>49</v>
-      </c>
-      <c r="I6" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -702,7 +713,7 @@
       <c r="C7" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" t="s">
         <v>28</v>
       </c>
       <c r="E7" t="s">
@@ -716,7 +727,7 @@
         <v>5</v>
       </c>
       <c r="H7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -726,7 +737,7 @@
       <c r="C8" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" t="s">
         <v>28</v>
       </c>
       <c r="E8" t="s">
@@ -746,7 +757,7 @@
       <c r="C9" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" t="s">
         <v>28</v>
       </c>
       <c r="E9" t="s">
@@ -766,7 +777,7 @@
       <c r="C10" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" t="s">
         <v>28</v>
       </c>
       <c r="E10" t="s">
@@ -786,7 +797,7 @@
       <c r="C11" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" t="s">
         <v>28</v>
       </c>
       <c r="E11" t="s">
@@ -809,8 +820,8 @@
       <c r="C13" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="18" t="s">
-        <v>44</v>
+      <c r="D13" t="s">
+        <v>43</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -823,7 +834,7 @@
         <v>5</v>
       </c>
       <c r="I13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -833,8 +844,8 @@
       <c r="C14" t="s">
         <v>36</v>
       </c>
-      <c r="D14" s="18" t="s">
-        <v>44</v>
+      <c r="D14" t="s">
+        <v>43</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -854,8 +865,8 @@
       <c r="C15" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="18" t="s">
-        <v>44</v>
+      <c r="D15" t="s">
+        <v>43</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -874,8 +885,8 @@
       <c r="C16" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="18" t="s">
-        <v>44</v>
+      <c r="D16" t="s">
+        <v>43</v>
       </c>
       <c r="E16" t="s">
         <v>10</v>
@@ -894,8 +905,8 @@
       <c r="C17" t="s">
         <v>29</v>
       </c>
-      <c r="D17" s="18" t="s">
-        <v>44</v>
+      <c r="D17" t="s">
+        <v>43</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
@@ -914,8 +925,8 @@
       <c r="C18" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="18" t="s">
-        <v>44</v>
+      <c r="D18" t="s">
+        <v>43</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -937,8 +948,8 @@
       <c r="C20" t="s">
         <v>29</v>
       </c>
-      <c r="D20" s="18" t="s">
-        <v>45</v>
+      <c r="D20" t="s">
+        <v>44</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -951,7 +962,7 @@
         <v>5</v>
       </c>
       <c r="I20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -961,8 +972,8 @@
       <c r="C21" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="18" t="s">
-        <v>45</v>
+      <c r="D21" t="s">
+        <v>44</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
@@ -982,8 +993,8 @@
       <c r="C22" t="s">
         <v>29</v>
       </c>
-      <c r="D22" s="18" t="s">
-        <v>45</v>
+      <c r="D22" t="s">
+        <v>44</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -1002,8 +1013,8 @@
       <c r="C23" t="s">
         <v>29</v>
       </c>
-      <c r="D23" s="18" t="s">
-        <v>45</v>
+      <c r="D23" t="s">
+        <v>44</v>
       </c>
       <c r="E23" t="s">
         <v>10</v>
@@ -1022,8 +1033,8 @@
       <c r="C24" t="s">
         <v>29</v>
       </c>
-      <c r="D24" s="18" t="s">
-        <v>45</v>
+      <c r="D24" t="s">
+        <v>44</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -1042,8 +1053,8 @@
       <c r="C25" t="s">
         <v>29</v>
       </c>
-      <c r="D25" s="18" t="s">
-        <v>45</v>
+      <c r="D25" t="s">
+        <v>44</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
@@ -1065,8 +1076,8 @@
       <c r="C27" t="s">
         <v>29</v>
       </c>
-      <c r="D27" s="18" t="s">
-        <v>47</v>
+      <c r="D27" t="s">
+        <v>46</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
@@ -1079,7 +1090,7 @@
         <v>5</v>
       </c>
       <c r="I27" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -1089,8 +1100,8 @@
       <c r="C28" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="18" t="s">
-        <v>47</v>
+      <c r="D28" t="s">
+        <v>46</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -1110,8 +1121,8 @@
       <c r="C29" t="s">
         <v>29</v>
       </c>
-      <c r="D29" s="18" t="s">
-        <v>47</v>
+      <c r="D29" t="s">
+        <v>46</v>
       </c>
       <c r="E29" t="s">
         <v>10</v>
@@ -1130,8 +1141,8 @@
       <c r="C30" t="s">
         <v>29</v>
       </c>
-      <c r="D30" s="18" t="s">
-        <v>47</v>
+      <c r="D30" t="s">
+        <v>46</v>
       </c>
       <c r="E30" t="s">
         <v>10</v>
@@ -1150,8 +1161,8 @@
       <c r="C31" t="s">
         <v>29</v>
       </c>
-      <c r="D31" s="18" t="s">
-        <v>47</v>
+      <c r="D31" t="s">
+        <v>46</v>
       </c>
       <c r="E31" t="s">
         <v>10</v>
@@ -1170,8 +1181,8 @@
       <c r="C32" t="s">
         <v>29</v>
       </c>
-      <c r="D32" s="18" t="s">
-        <v>47</v>
+      <c r="D32" t="s">
+        <v>46</v>
       </c>
       <c r="E32" t="s">
         <v>10</v>
@@ -1193,8 +1204,8 @@
       <c r="C34" t="s">
         <v>29</v>
       </c>
-      <c r="D34" s="18" t="s">
-        <v>46</v>
+      <c r="D34" t="s">
+        <v>45</v>
       </c>
       <c r="E34" t="s">
         <v>10</v>
@@ -1207,7 +1218,7 @@
         <v>5</v>
       </c>
       <c r="I34" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -1217,8 +1228,8 @@
       <c r="C35" t="s">
         <v>36</v>
       </c>
-      <c r="D35" s="18" t="s">
-        <v>46</v>
+      <c r="D35" t="s">
+        <v>45</v>
       </c>
       <c r="E35" t="s">
         <v>10</v>
@@ -1238,8 +1249,8 @@
       <c r="C36" t="s">
         <v>29</v>
       </c>
-      <c r="D36" s="18" t="s">
-        <v>46</v>
+      <c r="D36" t="s">
+        <v>45</v>
       </c>
       <c r="E36" t="s">
         <v>10</v>
@@ -1258,8 +1269,8 @@
       <c r="C37" t="s">
         <v>29</v>
       </c>
-      <c r="D37" s="18" t="s">
-        <v>46</v>
+      <c r="D37" t="s">
+        <v>45</v>
       </c>
       <c r="E37" t="s">
         <v>10</v>
@@ -1278,8 +1289,8 @@
       <c r="C38" t="s">
         <v>29</v>
       </c>
-      <c r="D38" s="18" t="s">
-        <v>46</v>
+      <c r="D38" t="s">
+        <v>45</v>
       </c>
       <c r="E38" t="s">
         <v>10</v>
@@ -1298,8 +1309,8 @@
       <c r="C39" t="s">
         <v>29</v>
       </c>
-      <c r="D39" s="18" t="s">
-        <v>46</v>
+      <c r="D39" t="s">
+        <v>45</v>
       </c>
       <c r="E39" t="s">
         <v>10</v>
@@ -1315,23 +1326,23 @@
       <c r="F40" s="2"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D41" s="18" t="s">
-        <v>42</v>
+      <c r="D41" t="s">
+        <v>41</v>
       </c>
       <c r="F41" s="2"/>
       <c r="H41" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D42" s="18" t="s">
-        <v>43</v>
+      <c r="D42" t="s">
+        <v>42</v>
       </c>
       <c r="F42" s="2"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D43" s="18" t="s">
-        <v>41</v>
+      <c r="D43" t="s">
+        <v>40</v>
       </c>
       <c r="F43" s="2"/>
     </row>
@@ -1577,42 +1588,51 @@
       <c r="I62" s="6"/>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A63" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="F63" s="15"/>
+      <c r="C63" t="s">
+        <v>29</v>
+      </c>
+      <c r="E63" t="s">
+        <v>15</v>
+      </c>
+      <c r="F63" s="15">
+        <f>43/100</f>
+        <v>0.43</v>
+      </c>
+      <c r="G63" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C64" t="s">
         <v>29</v>
       </c>
       <c r="E64" t="s">
-        <v>15</v>
-      </c>
-      <c r="F64" s="15">
-        <f>43/100</f>
+        <v>16</v>
+      </c>
+      <c r="F64" s="16">
+        <f>F63</f>
         <v>0.43</v>
       </c>
       <c r="G64" t="s">
         <v>19</v>
       </c>
+      <c r="H64" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C65" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="E65" t="s">
-        <v>16</v>
-      </c>
-      <c r="F65" s="16">
-        <f>F64</f>
-        <v>0.43</v>
+        <v>15</v>
+      </c>
+      <c r="F65" s="15">
+        <f>41/100</f>
+        <v>0.41</v>
       </c>
       <c r="G65" t="s">
         <v>19</v>
-      </c>
-      <c r="H65" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -1620,76 +1640,65 @@
         <v>36</v>
       </c>
       <c r="E66" t="s">
-        <v>15</v>
-      </c>
-      <c r="F66" s="15">
-        <f>41/100</f>
+        <v>16</v>
+      </c>
+      <c r="F66" s="16">
+        <f>F65</f>
         <v>0.41</v>
       </c>
       <c r="G66" t="s">
         <v>19</v>
       </c>
+      <c r="H66" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C67" t="s">
-        <v>36</v>
-      </c>
-      <c r="E67" t="s">
-        <v>16</v>
-      </c>
-      <c r="F67" s="16">
-        <f>F66</f>
-        <v>0.41</v>
-      </c>
-      <c r="G67" t="s">
-        <v>19</v>
-      </c>
-      <c r="H67" t="s">
-        <v>37</v>
-      </c>
+      <c r="F67" s="16"/>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F68" s="2"/>
+      <c r="E68" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="F68" s="13">
+        <v>0.65</v>
+      </c>
+      <c r="G68" t="s">
+        <v>56</v>
+      </c>
+      <c r="H68" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I68" s="9" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A69" s="8" t="s">
+      <c r="F69" s="2"/>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A70" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B69" s="8"/>
-      <c r="C69" s="6"/>
-      <c r="D69" s="8"/>
-      <c r="E69" s="6"/>
-      <c r="F69" s="7"/>
-      <c r="G69" s="6"/>
-      <c r="H69" s="6"/>
-      <c r="I69" s="6"/>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C70" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D70" s="9"/>
-      <c r="E70" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F70" s="10">
-        <v>0</v>
-      </c>
-      <c r="G70" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="H70" s="4"/>
+      <c r="B70" s="8"/>
+      <c r="C70" s="6"/>
+      <c r="D70" s="8"/>
+      <c r="E70" s="6"/>
+      <c r="F70" s="7"/>
+      <c r="G70" s="6"/>
+      <c r="H70" s="6"/>
+      <c r="I70" s="6"/>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C71" s="9" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D71" s="9"/>
       <c r="E71" s="9" t="s">
         <v>22</v>
       </c>
       <c r="F71" s="10">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G71" s="9" t="s">
         <v>23</v>
@@ -1697,32 +1706,40 @@
       <c r="H71" s="4"/>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F72" s="2"/>
+      <c r="C72" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D72" s="9"/>
+      <c r="E72" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F72" s="10">
+        <v>10</v>
+      </c>
+      <c r="G72" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="H72" s="4"/>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A73" s="8" t="s">
+      <c r="F73" s="2"/>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A74" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B73" s="8"/>
-      <c r="C73" s="6"/>
-      <c r="D73" s="8"/>
-      <c r="E73" s="6"/>
-      <c r="F73" s="7"/>
-      <c r="G73" s="6"/>
-      <c r="H73" s="6"/>
-      <c r="I73" s="6"/>
-    </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A74" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B74" s="3"/>
-      <c r="D74" s="3"/>
-      <c r="F74" s="2"/>
+      <c r="B74" s="8"/>
+      <c r="C74" s="6"/>
+      <c r="D74" s="8"/>
+      <c r="E74" s="6"/>
+      <c r="F74" s="7"/>
+      <c r="G74" s="6"/>
+      <c r="H74" s="6"/>
+      <c r="I74" s="6"/>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B75" s="3"/>
       <c r="D75" s="3"/>
@@ -1730,35 +1747,26 @@
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B76" s="3"/>
       <c r="D76" s="3"/>
       <c r="F76" s="2"/>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A77" s="3"/>
+      <c r="A77" s="3" t="s">
+        <v>54</v>
+      </c>
       <c r="B77" s="3"/>
       <c r="D77" s="3"/>
-      <c r="E77" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F77" s="5">
-        <v>1</v>
-      </c>
-      <c r="G77" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H77" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="F77" s="2"/>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="D78" s="3"/>
       <c r="E78" s="4" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="F78" s="5">
         <v>1</v>
@@ -1774,30 +1782,31 @@
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="D79" s="3"/>
-      <c r="E79" s="4"/>
-      <c r="F79" s="5"/>
-      <c r="G79" s="4"/>
-      <c r="H79" s="4"/>
+      <c r="E79" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F79" s="5">
+        <v>1</v>
+      </c>
+      <c r="G79" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H79" s="4" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C80" t="s">
-        <v>29</v>
-      </c>
-      <c r="E80" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F80" s="13">
-        <f>1-0.43</f>
-        <v>0.57000000000000006</v>
-      </c>
-      <c r="G80" s="9" t="s">
-        <v>26</v>
-      </c>
+      <c r="A80" s="3"/>
+      <c r="B80" s="3"/>
+      <c r="D80" s="3"/>
+      <c r="E80" s="4"/>
+      <c r="F80" s="5"/>
+      <c r="G80" s="4"/>
       <c r="H80" s="4"/>
     </row>
-    <row r="81" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C81" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>25</v>
@@ -1809,72 +1818,85 @@
       <c r="G81" s="9" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="82" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="F82" s="2"/>
-    </row>
-    <row r="83" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C83" t="s">
-        <v>29</v>
-      </c>
-      <c r="E83" t="s">
-        <v>53</v>
-      </c>
-      <c r="F83" s="12">
+      <c r="H81" s="4"/>
+    </row>
+    <row r="82" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C82" t="s">
+        <v>36</v>
+      </c>
+      <c r="E82" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F82" s="13">
+        <f>1-0.43</f>
+        <v>0.57000000000000006</v>
+      </c>
+      <c r="G82" s="9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="83" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="F83" s="2"/>
+    </row>
+    <row r="84" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C84" t="s">
+        <v>29</v>
+      </c>
+      <c r="E84" t="s">
+        <v>52</v>
+      </c>
+      <c r="F84" s="12">
         <v>0.5</v>
-      </c>
-      <c r="G83" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="84" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C84" t="s">
-        <v>36</v>
-      </c>
-      <c r="E84" t="s">
-        <v>53</v>
-      </c>
-      <c r="F84" s="12">
-        <v>1</v>
       </c>
       <c r="G84" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="85" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="F85" s="2"/>
-    </row>
-    <row r="86" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C85" t="s">
+        <v>36</v>
+      </c>
+      <c r="E85" t="s">
+        <v>52</v>
+      </c>
+      <c r="F85" s="12">
+        <v>1</v>
+      </c>
+      <c r="G85" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="86" spans="3:8" x14ac:dyDescent="0.25">
       <c r="F86" s="2"/>
     </row>
-    <row r="87" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="3:8" x14ac:dyDescent="0.25">
       <c r="F87" s="2"/>
     </row>
-    <row r="88" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="3:8" x14ac:dyDescent="0.25">
       <c r="F88" s="2"/>
     </row>
-    <row r="89" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="3:8" x14ac:dyDescent="0.25">
       <c r="F89" s="2"/>
     </row>
-    <row r="90" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="3:8" x14ac:dyDescent="0.25">
       <c r="F90" s="2"/>
     </row>
-    <row r="91" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="3:8" x14ac:dyDescent="0.25">
       <c r="F91" s="2"/>
     </row>
-    <row r="92" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="3:8" x14ac:dyDescent="0.25">
       <c r="F92" s="2"/>
     </row>
-    <row r="93" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="3:8" x14ac:dyDescent="0.25">
       <c r="F93" s="2"/>
     </row>
-    <row r="94" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="3:8" x14ac:dyDescent="0.25">
       <c r="F94" s="2"/>
     </row>
-    <row r="95" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="3:8" x14ac:dyDescent="0.25">
       <c r="F95" s="2"/>
     </row>
-    <row r="96" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="3:8" x14ac:dyDescent="0.25">
       <c r="F96" s="2"/>
     </row>
     <row r="97" spans="6:6" x14ac:dyDescent="0.25">
@@ -1936,6 +1958,9 @@
     </row>
     <row r="116" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F116" s="2"/>
+    </row>
+    <row r="117" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F117" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>